<commit_message>
Refresh FEC data 2026-09-28 23:33 UTC
</commit_message>
<xml_diff>
--- a/site/PA07_Campaign_Finance.xlsx
+++ b/site/PA07_Campaign_Finance.xlsx
@@ -3607,7 +3607,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>2026-09-24T15:07:26Z</t>
+          <t>2026-09-28T23:32:20Z</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -4176,7 +4176,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Final full-cycle FEC totals and certified vote totals. One row per nominee per election. Retrieved 2026-09-17T15:59:59Z.</t>
+          <t>Final full-cycle FEC totals and certified vote totals. One row per nominee per election. Retrieved 2026-09-28T23:33:30Z.</t>
         </is>
       </c>
     </row>
@@ -6444,14 +6444,14 @@
     <row r="4" ht="120" customHeight="1">
       <c r="A4" s="85" t="inlineStr">
         <is>
-          <t>Current cycle: FEC / OpenFEC API, https://www.fec.gov/data/elections/house/PA/07/2026/, retrieved 2026-09-24T15:07:26Z</t>
+          <t>Current cycle: FEC / OpenFEC API, https://www.fec.gov/data/elections/house/PA/07/2026/, retrieved 2026-09-28T23:32:20Z</t>
         </is>
       </c>
     </row>
     <row r="5" ht="108" customHeight="1">
       <c r="A5" s="85" t="inlineStr">
         <is>
-          <t>History, finance: OpenFEC API (finance); certified results from sources/results.json, retrieved 2026-09-17T15:59:59Z</t>
+          <t>History, finance: OpenFEC API (finance); certified results from sources/results.json, retrieved 2026-09-28T23:33:30Z</t>
         </is>
       </c>
     </row>
@@ -29499,7 +29499,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cycle-to-date from each committee's latest periodic FEC report. Coverage through 2026-06-30. Retrieved 2026-09-24T15:07:26Z.</t>
+          <t>Cycle-to-date from each committee's latest periodic FEC report. Coverage through 2026-06-30. Retrieved 2026-09-28T23:32:20Z.</t>
         </is>
       </c>
     </row>
@@ -31158,7 +31158,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Itemized disbursements (each over $200), 2026 cycle, through 2026-06-30. Categories assigned from the description on each report. Retrieved 2026-09-18T01:21:30Z.</t>
+          <t>Itemized disbursements (each over $200), 2026 cycle, through 2026-06-30. Categories assigned from the description on each report. Retrieved 2026-09-28T23:33:24Z.</t>
         </is>
       </c>
     </row>
@@ -32950,7 +32950,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Itemized individual contributions (each over $200), 2026 cycle, through 2026-06-30. FEC aggregates. Retrieved 2026-09-18T01:21:30Z.</t>
+          <t>Itemized individual contributions (each over $200), 2026 cycle, through 2026-06-30. FEC aggregates. Retrieved 2026-09-28T23:33:24Z.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh FEC data 2026-10-15 12:00 UTC
</commit_message>
<xml_diff>
--- a/site/PA07_Campaign_Finance.xlsx
+++ b/site/PA07_Campaign_Finance.xlsx
@@ -3573,7 +3573,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -3607,7 +3607,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>2026-10-09T17:05:35Z</t>
+          <t>2026-10-15T11:59:42Z</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -6444,7 +6444,7 @@
     <row r="4" ht="120" customHeight="1">
       <c r="A4" s="85" t="inlineStr">
         <is>
-          <t>Current cycle: FEC / OpenFEC API, https://www.fec.gov/data/elections/house/PA/07/2026/, retrieved 2026-10-09T17:05:35Z</t>
+          <t>Current cycle: FEC / OpenFEC API, https://www.fec.gov/data/elections/house/PA/07/2026/, retrieved 2026-10-15T11:59:42Z</t>
         </is>
       </c>
     </row>
@@ -14900,7 +14900,7 @@
       </c>
       <c r="M168" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -14941,7 +14941,7 @@
       </c>
       <c r="M169" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -14982,7 +14982,7 @@
       </c>
       <c r="M170" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15023,7 +15023,7 @@
       </c>
       <c r="M171" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15064,7 +15064,7 @@
       </c>
       <c r="M172" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15105,7 +15105,7 @@
       </c>
       <c r="M173" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15146,7 +15146,7 @@
       </c>
       <c r="M174" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15187,7 +15187,7 @@
       </c>
       <c r="M175" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15228,7 +15228,7 @@
       </c>
       <c r="M176" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15269,7 +15269,7 @@
       </c>
       <c r="M177" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15310,7 +15310,7 @@
       </c>
       <c r="M178" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15351,7 +15351,7 @@
       </c>
       <c r="M179" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15392,7 +15392,7 @@
       </c>
       <c r="M180" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15433,7 +15433,7 @@
       </c>
       <c r="M181" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15474,7 +15474,7 @@
       </c>
       <c r="M182" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15515,7 +15515,7 @@
       </c>
       <c r="M183" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15568,7 +15568,7 @@
       </c>
       <c r="M184" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15621,7 +15621,7 @@
       </c>
       <c r="M185" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15674,7 +15674,7 @@
       </c>
       <c r="M186" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15727,7 +15727,7 @@
       </c>
       <c r="M187" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15780,7 +15780,7 @@
       </c>
       <c r="M188" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15833,7 +15833,7 @@
       </c>
       <c r="M189" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15886,7 +15886,7 @@
       </c>
       <c r="M190" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15939,7 +15939,7 @@
       </c>
       <c r="M191" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -15992,7 +15992,7 @@
       </c>
       <c r="M192" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16045,7 +16045,7 @@
       </c>
       <c r="M193" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16098,7 +16098,7 @@
       </c>
       <c r="M194" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16151,7 +16151,7 @@
       </c>
       <c r="M195" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16204,7 +16204,7 @@
       </c>
       <c r="M196" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16257,7 +16257,7 @@
       </c>
       <c r="M197" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16310,7 +16310,7 @@
       </c>
       <c r="M198" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16351,7 +16351,7 @@
       </c>
       <c r="M199" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16392,7 +16392,7 @@
       </c>
       <c r="M200" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16433,7 +16433,7 @@
       </c>
       <c r="M201" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16474,7 +16474,7 @@
       </c>
       <c r="M202" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16515,7 +16515,7 @@
       </c>
       <c r="M203" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16556,7 +16556,7 @@
       </c>
       <c r="M204" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="M205" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16638,7 +16638,7 @@
       </c>
       <c r="M206" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16679,7 +16679,7 @@
       </c>
       <c r="M207" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16720,7 +16720,7 @@
       </c>
       <c r="M208" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16761,7 +16761,7 @@
       </c>
       <c r="M209" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16802,7 +16802,7 @@
       </c>
       <c r="M210" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16843,7 +16843,7 @@
       </c>
       <c r="M211" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16884,7 +16884,7 @@
       </c>
       <c r="M212" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16925,7 +16925,7 @@
       </c>
       <c r="M213" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -16966,7 +16966,7 @@
       </c>
       <c r="M214" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17007,7 +17007,7 @@
       </c>
       <c r="M215" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17048,7 +17048,7 @@
       </c>
       <c r="M216" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17089,7 +17089,7 @@
       </c>
       <c r="M217" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17130,7 +17130,7 @@
       </c>
       <c r="M218" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17171,7 +17171,7 @@
       </c>
       <c r="M219" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17212,7 +17212,7 @@
       </c>
       <c r="M220" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17253,7 +17253,7 @@
       </c>
       <c r="M221" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17294,7 +17294,7 @@
       </c>
       <c r="M222" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17335,7 +17335,7 @@
       </c>
       <c r="M223" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17376,7 +17376,7 @@
       </c>
       <c r="M224" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17417,7 +17417,7 @@
       </c>
       <c r="M225" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17458,7 +17458,7 @@
       </c>
       <c r="M226" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17499,7 +17499,7 @@
       </c>
       <c r="M227" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17540,7 +17540,7 @@
       </c>
       <c r="M228" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17581,7 +17581,7 @@
       </c>
       <c r="M229" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17622,7 +17622,7 @@
       </c>
       <c r="M230" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17663,7 +17663,7 @@
       </c>
       <c r="M231" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17704,7 +17704,7 @@
       </c>
       <c r="M232" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17745,7 +17745,7 @@
       </c>
       <c r="M233" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17786,7 +17786,7 @@
       </c>
       <c r="M234" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17827,7 +17827,7 @@
       </c>
       <c r="M235" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17868,7 +17868,7 @@
       </c>
       <c r="M236" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17909,7 +17909,7 @@
       </c>
       <c r="M237" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17950,7 +17950,7 @@
       </c>
       <c r="M238" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -17991,7 +17991,7 @@
       </c>
       <c r="M239" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18032,7 +18032,7 @@
       </c>
       <c r="M240" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18073,7 +18073,7 @@
       </c>
       <c r="M241" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18114,7 +18114,7 @@
       </c>
       <c r="M242" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18155,7 +18155,7 @@
       </c>
       <c r="M243" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18196,7 +18196,7 @@
       </c>
       <c r="M244" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18237,7 +18237,7 @@
       </c>
       <c r="M245" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18278,7 +18278,7 @@
       </c>
       <c r="M246" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18319,7 +18319,7 @@
       </c>
       <c r="M247" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18360,7 +18360,7 @@
       </c>
       <c r="M248" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18401,7 +18401,7 @@
       </c>
       <c r="M249" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18442,7 +18442,7 @@
       </c>
       <c r="M250" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18483,7 +18483,7 @@
       </c>
       <c r="M251" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18524,7 +18524,7 @@
       </c>
       <c r="M252" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18565,7 +18565,7 @@
       </c>
       <c r="M253" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18606,7 +18606,7 @@
       </c>
       <c r="M254" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18647,7 +18647,7 @@
       </c>
       <c r="M255" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18688,7 +18688,7 @@
       </c>
       <c r="M256" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18729,7 +18729,7 @@
       </c>
       <c r="M257" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18770,7 +18770,7 @@
       </c>
       <c r="M258" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18811,7 +18811,7 @@
       </c>
       <c r="M259" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18852,7 +18852,7 @@
       </c>
       <c r="M260" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18893,7 +18893,7 @@
       </c>
       <c r="M261" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18934,7 +18934,7 @@
       </c>
       <c r="M262" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -18973,7 +18973,7 @@
       <c r="L263" s="34" t="n"/>
       <c r="M263" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19014,7 +19014,7 @@
       </c>
       <c r="M264" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19055,7 +19055,7 @@
       </c>
       <c r="M265" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19096,7 +19096,7 @@
       </c>
       <c r="M266" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19137,7 +19137,7 @@
       </c>
       <c r="M267" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19180,7 +19180,7 @@
       <c r="L268" s="34" t="n"/>
       <c r="M268" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19221,7 +19221,7 @@
       </c>
       <c r="M269" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19262,7 +19262,7 @@
       </c>
       <c r="M270" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19303,7 +19303,7 @@
       </c>
       <c r="M271" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19344,7 +19344,7 @@
       </c>
       <c r="M272" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19385,7 +19385,7 @@
       </c>
       <c r="M273" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19426,7 +19426,7 @@
       </c>
       <c r="M274" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19467,7 +19467,7 @@
       </c>
       <c r="M275" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19508,7 +19508,7 @@
       </c>
       <c r="M276" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19549,7 @@
       </c>
       <c r="M277" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19590,7 +19590,7 @@
       </c>
       <c r="M278" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19631,7 +19631,7 @@
       </c>
       <c r="M279" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19672,7 +19672,7 @@
       </c>
       <c r="M280" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19713,7 +19713,7 @@
       </c>
       <c r="M281" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19754,7 +19754,7 @@
       </c>
       <c r="M282" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19795,7 +19795,7 @@
       </c>
       <c r="M283" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19836,7 +19836,7 @@
       </c>
       <c r="M284" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19877,7 +19877,7 @@
       </c>
       <c r="M285" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19918,7 +19918,7 @@
       </c>
       <c r="M286" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -19959,7 +19959,7 @@
       </c>
       <c r="M287" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20000,7 +20000,7 @@
       </c>
       <c r="M288" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20041,7 +20041,7 @@
       </c>
       <c r="M289" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20082,7 +20082,7 @@
       </c>
       <c r="M290" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20123,7 +20123,7 @@
       </c>
       <c r="M291" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20164,7 +20164,7 @@
       </c>
       <c r="M292" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20205,7 +20205,7 @@
       </c>
       <c r="M293" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20246,7 +20246,7 @@
       </c>
       <c r="M294" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20287,7 +20287,7 @@
       </c>
       <c r="M295" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20328,7 +20328,7 @@
       </c>
       <c r="M296" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20369,7 +20369,7 @@
       </c>
       <c r="M297" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20410,7 +20410,7 @@
       </c>
       <c r="M298" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20451,7 +20451,7 @@
       </c>
       <c r="M299" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20492,7 +20492,7 @@
       </c>
       <c r="M300" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20533,7 +20533,7 @@
       </c>
       <c r="M301" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20574,7 +20574,7 @@
       </c>
       <c r="M302" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20615,7 +20615,7 @@
       </c>
       <c r="M303" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20656,7 +20656,7 @@
       </c>
       <c r="M304" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20697,7 +20697,7 @@
       </c>
       <c r="M305" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20738,7 +20738,7 @@
       </c>
       <c r="M306" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20791,7 +20791,7 @@
       </c>
       <c r="M307" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20844,7 +20844,7 @@
       </c>
       <c r="M308" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20897,7 +20897,7 @@
       </c>
       <c r="M309" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -20950,7 +20950,7 @@
       </c>
       <c r="M310" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21003,7 +21003,7 @@
       </c>
       <c r="M311" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21056,7 +21056,7 @@
       </c>
       <c r="M312" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21109,7 +21109,7 @@
       </c>
       <c r="M313" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21162,7 +21162,7 @@
       </c>
       <c r="M314" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21215,7 +21215,7 @@
       </c>
       <c r="M315" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21268,7 +21268,7 @@
       </c>
       <c r="M316" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21321,7 +21321,7 @@
       </c>
       <c r="M317" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="M318" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21427,7 +21427,7 @@
       </c>
       <c r="M319" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21480,7 +21480,7 @@
       </c>
       <c r="M320" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21533,7 +21533,7 @@
       </c>
       <c r="M321" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21574,7 +21574,7 @@
       </c>
       <c r="M322" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21615,7 +21615,7 @@
       </c>
       <c r="M323" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21656,7 +21656,7 @@
       </c>
       <c r="M324" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21697,7 +21697,7 @@
       </c>
       <c r="M325" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21738,7 +21738,7 @@
       </c>
       <c r="M326" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21779,7 +21779,7 @@
       </c>
       <c r="M327" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21820,7 +21820,7 @@
       </c>
       <c r="M328" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21861,7 +21861,7 @@
       </c>
       <c r="M329" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21902,7 +21902,7 @@
       </c>
       <c r="M330" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21943,7 +21943,7 @@
       </c>
       <c r="M331" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -21984,7 +21984,7 @@
       </c>
       <c r="M332" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22025,7 +22025,7 @@
       </c>
       <c r="M333" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22066,7 +22066,7 @@
       </c>
       <c r="M334" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22107,7 +22107,7 @@
       </c>
       <c r="M335" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22148,7 +22148,7 @@
       </c>
       <c r="M336" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22189,7 +22189,7 @@
       </c>
       <c r="M337" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22230,7 +22230,7 @@
       </c>
       <c r="M338" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22271,7 +22271,7 @@
       </c>
       <c r="M339" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22312,7 +22312,7 @@
       </c>
       <c r="M340" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22353,7 +22353,7 @@
       </c>
       <c r="M341" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22394,7 +22394,7 @@
       </c>
       <c r="M342" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22435,7 +22435,7 @@
       </c>
       <c r="M343" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22476,7 +22476,7 @@
       </c>
       <c r="M344" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22517,7 +22517,7 @@
       </c>
       <c r="M345" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22558,7 +22558,7 @@
       </c>
       <c r="M346" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22599,7 +22599,7 @@
       </c>
       <c r="M347" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22640,7 +22640,7 @@
       </c>
       <c r="M348" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22681,7 +22681,7 @@
       </c>
       <c r="M349" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22722,7 +22722,7 @@
       </c>
       <c r="M350" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22763,7 +22763,7 @@
       </c>
       <c r="M351" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22804,7 +22804,7 @@
       </c>
       <c r="M352" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22845,7 +22845,7 @@
       </c>
       <c r="M353" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22886,7 +22886,7 @@
       </c>
       <c r="M354" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22927,7 +22927,7 @@
       </c>
       <c r="M355" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -22968,7 +22968,7 @@
       </c>
       <c r="M356" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23009,7 +23009,7 @@
       </c>
       <c r="M357" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23050,7 +23050,7 @@
       </c>
       <c r="M358" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23091,7 +23091,7 @@
       </c>
       <c r="M359" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23132,7 +23132,7 @@
       </c>
       <c r="M360" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23173,7 +23173,7 @@
       </c>
       <c r="M361" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23214,7 +23214,7 @@
       </c>
       <c r="M362" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23255,7 +23255,7 @@
       </c>
       <c r="M363" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23296,7 +23296,7 @@
       </c>
       <c r="M364" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23337,7 +23337,7 @@
       </c>
       <c r="M365" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23378,7 +23378,7 @@
       </c>
       <c r="M366" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23419,7 +23419,7 @@
       </c>
       <c r="M367" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23460,7 +23460,7 @@
       </c>
       <c r="M368" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23501,7 +23501,7 @@
       </c>
       <c r="M369" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23542,7 +23542,7 @@
       </c>
       <c r="M370" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23583,7 +23583,7 @@
       </c>
       <c r="M371" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23624,7 +23624,7 @@
       </c>
       <c r="M372" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23665,7 +23665,7 @@
       </c>
       <c r="M373" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23706,7 +23706,7 @@
       </c>
       <c r="M374" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23747,7 +23747,7 @@
       </c>
       <c r="M375" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23788,7 +23788,7 @@
       </c>
       <c r="M376" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23829,7 +23829,7 @@
       </c>
       <c r="M377" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23870,7 +23870,7 @@
       </c>
       <c r="M378" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23911,7 +23911,7 @@
       </c>
       <c r="M379" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23952,7 +23952,7 @@
       </c>
       <c r="M380" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -23993,7 +23993,7 @@
       </c>
       <c r="M381" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24034,7 +24034,7 @@
       </c>
       <c r="M382" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24075,7 +24075,7 @@
       </c>
       <c r="M383" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24116,7 +24116,7 @@
       </c>
       <c r="M384" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24157,7 +24157,7 @@
       </c>
       <c r="M385" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24198,7 +24198,7 @@
       </c>
       <c r="M386" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24239,7 +24239,7 @@
       </c>
       <c r="M387" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24280,7 +24280,7 @@
       </c>
       <c r="M388" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24321,7 +24321,7 @@
       </c>
       <c r="M389" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24362,7 +24362,7 @@
       </c>
       <c r="M390" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24403,7 +24403,7 @@
       </c>
       <c r="M391" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24444,7 +24444,7 @@
       </c>
       <c r="M392" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24485,7 +24485,7 @@
       </c>
       <c r="M393" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24526,7 +24526,7 @@
       </c>
       <c r="M394" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24567,7 +24567,7 @@
       </c>
       <c r="M395" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24608,7 +24608,7 @@
       </c>
       <c r="M396" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24649,7 +24649,7 @@
       </c>
       <c r="M397" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24690,7 +24690,7 @@
       </c>
       <c r="M398" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24731,7 +24731,7 @@
       </c>
       <c r="M399" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24772,7 +24772,7 @@
       </c>
       <c r="M400" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24811,7 +24811,7 @@
       <c r="L401" s="34" t="n"/>
       <c r="M401" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24852,7 +24852,7 @@
       </c>
       <c r="M402" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24893,7 +24893,7 @@
       </c>
       <c r="M403" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24934,7 +24934,7 @@
       </c>
       <c r="M404" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -24975,7 +24975,7 @@
       </c>
       <c r="M405" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25018,7 +25018,7 @@
       <c r="L406" s="34" t="n"/>
       <c r="M406" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25059,7 +25059,7 @@
       </c>
       <c r="M407" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25100,7 +25100,7 @@
       </c>
       <c r="M408" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25141,7 +25141,7 @@
       </c>
       <c r="M409" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25182,7 +25182,7 @@
       </c>
       <c r="M410" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25223,7 +25223,7 @@
       </c>
       <c r="M411" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25264,7 +25264,7 @@
       </c>
       <c r="M412" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25305,7 +25305,7 @@
       </c>
       <c r="M413" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25346,7 +25346,7 @@
       </c>
       <c r="M414" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25387,7 +25387,7 @@
       </c>
       <c r="M415" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25428,7 +25428,7 @@
       </c>
       <c r="M416" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25469,7 +25469,7 @@
       </c>
       <c r="M417" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25510,7 +25510,7 @@
       </c>
       <c r="M418" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25551,7 +25551,7 @@
       </c>
       <c r="M419" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25592,7 +25592,7 @@
       </c>
       <c r="M420" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25633,7 +25633,7 @@
       </c>
       <c r="M421" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25674,7 +25674,7 @@
       </c>
       <c r="M422" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25715,7 +25715,7 @@
       </c>
       <c r="M423" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25756,7 +25756,7 @@
       </c>
       <c r="M424" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25797,7 +25797,7 @@
       </c>
       <c r="M425" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25838,7 +25838,7 @@
       </c>
       <c r="M426" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25879,7 +25879,7 @@
       </c>
       <c r="M427" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25920,7 +25920,7 @@
       </c>
       <c r="M428" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -25961,7 +25961,7 @@
       </c>
       <c r="M429" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -30096,7 +30096,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cycle-to-date from each committee's latest periodic FEC report. Coverage through 2026-06-30. Retrieved 2026-10-09T17:05:35Z.</t>
+          <t>Cycle-to-date from each committee's latest periodic FEC report. Coverage through 2026-09-30. Retrieved 2026-10-15T11:59:42Z.</t>
         </is>
       </c>
     </row>
@@ -31787,7 +31787,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Itemized disbursements (each over $200), 2026 cycle, through 2026-06-30. Categories assigned from the description on each report. Retrieved 2026-10-09T17:06:16Z.</t>
+          <t>Itemized disbursements (each over $200), 2026 cycle, through 2026-09-30. Categories assigned from the description on each report. Retrieved 2026-10-15T12:00:17Z.</t>
         </is>
       </c>
     </row>
@@ -33579,7 +33579,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Itemized individual contributions (each over $200), 2026 cycle, through 2026-06-30. FEC aggregates. Retrieved 2026-10-09T17:06:16Z.</t>
+          <t>Itemized individual contributions (each over $200), 2026 cycle, through 2026-09-30. FEC aggregates. Retrieved 2026-10-15T12:00:17Z.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh FEC data 2026-10-16 14:14 UTC
</commit_message>
<xml_diff>
--- a/site/PA07_Campaign_Finance.xlsx
+++ b/site/PA07_Campaign_Finance.xlsx
@@ -3607,7 +3607,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>2026-10-15T11:59:42Z</t>
+          <t>2026-10-16T14:14:36Z</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -6444,7 +6444,7 @@
     <row r="4" ht="120" customHeight="1">
       <c r="A4" s="85" t="inlineStr">
         <is>
-          <t>Current cycle: FEC / OpenFEC API, https://www.fec.gov/data/elections/house/PA/07/2026/, retrieved 2026-10-15T11:59:42Z</t>
+          <t>Current cycle: FEC / OpenFEC API, https://www.fec.gov/data/elections/house/PA/07/2026/, retrieved 2026-10-16T14:14:36Z</t>
         </is>
       </c>
     </row>
@@ -6838,12 +6838,12 @@
       <c r="I5" s="5" t="n"/>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="33" t="n">
-        <v>2392215.23</v>
+        <v>4991635.39</v>
       </c>
       <c r="L5" s="34" t="n"/>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -6877,12 +6877,12 @@
       <c r="I6" s="5" t="n"/>
       <c r="J6" s="5" t="n"/>
       <c r="K6" s="33" t="n">
-        <v>1373792.39</v>
+        <v>3705480.38</v>
       </c>
       <c r="L6" s="34" t="n"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -6916,12 +6916,12 @@
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="33" t="n">
-        <v>1018422.84</v>
+        <v>1286155.01</v>
       </c>
       <c r="L7" s="34" t="n"/>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       <c r="L8" s="34" t="n"/>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -6994,12 +6994,12 @@
       <c r="I9" s="5" t="n"/>
       <c r="J9" s="5" t="n"/>
       <c r="K9" s="33" t="n">
-        <v>1942165.53</v>
+        <v>3916290.29</v>
       </c>
       <c r="L9" s="34" t="n"/>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7033,12 +7033,12 @@
       <c r="I10" s="5" t="n"/>
       <c r="J10" s="5" t="n"/>
       <c r="K10" s="33" t="n">
-        <v>1342778.75</v>
+        <v>2848797.27</v>
       </c>
       <c r="L10" s="34" t="n"/>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7072,12 +7072,12 @@
       <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="n"/>
       <c r="K11" s="33" t="n">
-        <v>599386.78</v>
+        <v>1067493.02</v>
       </c>
       <c r="L11" s="34" t="n"/>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7111,12 +7111,12 @@
       <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
       <c r="K12" s="33" t="n">
-        <v>403000.03</v>
+        <v>596250.03</v>
       </c>
       <c r="L12" s="34" t="n"/>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7150,12 +7150,12 @@
       <c r="I13" s="5" t="n"/>
       <c r="J13" s="5" t="n"/>
       <c r="K13" s="33" t="n">
-        <v>5000</v>
+        <v>6090.07</v>
       </c>
       <c r="L13" s="34" t="n"/>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7189,12 +7189,12 @@
       <c r="I14" s="5" t="n"/>
       <c r="J14" s="5" t="n"/>
       <c r="K14" s="33" t="n">
-        <v>26085</v>
+        <v>456989.33</v>
       </c>
       <c r="L14" s="34" t="n"/>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7233,7 +7233,7 @@
       <c r="L15" s="34" t="n"/>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7267,12 +7267,12 @@
       <c r="I16" s="5" t="n"/>
       <c r="J16" s="5" t="n"/>
       <c r="K16" s="33" t="n">
-        <v>4357405.11</v>
+        <v>5167022.85</v>
       </c>
       <c r="L16" s="34" t="n"/>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7306,12 +7306,12 @@
       <c r="I17" s="5" t="n"/>
       <c r="J17" s="5" t="n"/>
       <c r="K17" s="33" t="n">
-        <v>1521927.85</v>
+        <v>3094595.78</v>
       </c>
       <c r="L17" s="34" t="n"/>
       <c r="M17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7345,12 +7345,12 @@
       <c r="I18" s="5" t="n"/>
       <c r="J18" s="5" t="n"/>
       <c r="K18" s="33" t="n">
-        <v>2938717.17</v>
+        <v>2175666.98</v>
       </c>
       <c r="L18" s="34" t="n"/>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7384,12 +7384,12 @@
       <c r="I19" s="5" t="n"/>
       <c r="J19" s="5" t="n"/>
       <c r="K19" s="33" t="n">
-        <v>22583.23</v>
+        <v>4184.82</v>
       </c>
       <c r="L19" s="34" t="n"/>
       <c r="M19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7423,12 +7423,12 @@
       <c r="I20" s="5" t="n"/>
       <c r="J20" s="5" t="n"/>
       <c r="K20" s="33" t="n">
-        <v>1493241.01</v>
+        <v>1840430.27</v>
       </c>
       <c r="L20" s="34" t="n"/>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7462,12 +7462,12 @@
       <c r="I21" s="5" t="n"/>
       <c r="J21" s="5" t="n"/>
       <c r="K21" s="33" t="n">
-        <v>939107.04</v>
+        <v>1191087.7</v>
       </c>
       <c r="L21" s="34" t="n"/>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7501,12 +7501,12 @@
       <c r="I22" s="5" t="n"/>
       <c r="J22" s="5" t="n"/>
       <c r="K22" s="33" t="n">
-        <v>554133.97</v>
+        <v>649342.5699999999</v>
       </c>
       <c r="L22" s="34" t="n"/>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7540,12 +7540,12 @@
       <c r="I23" s="5" t="n"/>
       <c r="J23" s="5" t="n"/>
       <c r="K23" s="33" t="n">
-        <v>1042912.78</v>
+        <v>1284212.78</v>
       </c>
       <c r="L23" s="34" t="n"/>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7579,12 +7579,12 @@
       <c r="I24" s="5" t="n"/>
       <c r="J24" s="5" t="n"/>
       <c r="K24" s="33" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="L24" s="34" t="n"/>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7618,12 +7618,12 @@
       <c r="I25" s="5" t="n"/>
       <c r="J25" s="5" t="n"/>
       <c r="K25" s="33" t="n">
-        <v>1779199.14</v>
+        <v>1982987.65</v>
       </c>
       <c r="L25" s="34" t="n"/>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -7662,7 +7662,7 @@
       <c r="L26" s="34" t="n"/>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -30096,7 +30096,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cycle-to-date from each committee's latest periodic FEC report. Coverage through 2026-09-30. Retrieved 2026-10-15T11:59:42Z.</t>
+          <t>Cycle-to-date from each committee's latest periodic FEC report. Coverage through 2026-09-30. Retrieved 2026-10-16T14:14:36Z.</t>
         </is>
       </c>
     </row>
@@ -30238,35 +30238,35 @@
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G6" s="44" t="n">
-        <v>4357405.11</v>
+        <v>5167022.85</v>
       </c>
       <c r="H6" s="44" t="n">
-        <v>1521927.85</v>
+        <v>3094595.78</v>
       </c>
       <c r="I6" s="44" t="n">
-        <v>2938717.17</v>
+        <v>2175666.98</v>
       </c>
       <c r="J6" s="44" t="n">
-        <v>22583.23</v>
+        <v>4184.82</v>
       </c>
       <c r="K6" s="44" t="n">
-        <v>1493241.01</v>
+        <v>1840430.27</v>
       </c>
       <c r="L6" s="44" t="n">
-        <v>554133.97</v>
+        <v>649342.5699999999</v>
       </c>
       <c r="M6" s="44" t="n">
-        <v>1042912.78</v>
+        <v>1284212.78</v>
       </c>
       <c r="N6" s="44" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="O6" s="44" t="n">
-        <v>1779199.14</v>
+        <v>1982987.65</v>
       </c>
       <c r="P6" s="44" t="n">
         <v>0</v>
@@ -30304,35 +30304,35 @@
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G7" s="44" t="n">
-        <v>2392215.23</v>
+        <v>4991635.39</v>
       </c>
       <c r="H7" s="44" t="n">
-        <v>1373792.39</v>
+        <v>3705480.38</v>
       </c>
       <c r="I7" s="44" t="n">
-        <v>1018422.84</v>
+        <v>1286155.01</v>
       </c>
       <c r="J7" s="44" t="n">
         <v>15000</v>
       </c>
       <c r="K7" s="44" t="n">
-        <v>1942165.53</v>
+        <v>3916290.29</v>
       </c>
       <c r="L7" s="44" t="n">
-        <v>599386.78</v>
+        <v>1067493.02</v>
       </c>
       <c r="M7" s="44" t="n">
-        <v>403000.03</v>
+        <v>596250.03</v>
       </c>
       <c r="N7" s="44" t="n">
-        <v>5000</v>
+        <v>6090.07</v>
       </c>
       <c r="O7" s="44" t="n">
-        <v>26085</v>
+        <v>456989.33</v>
       </c>
       <c r="P7" s="44" t="n">
         <v>3500</v>

</xml_diff>

<commit_message>
Refresh FEC data 2026-10-17 13:10 UTC
</commit_message>
<xml_diff>
--- a/site/PA07_Campaign_Finance.xlsx
+++ b/site/PA07_Campaign_Finance.xlsx
@@ -3607,7 +3607,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>2026-10-16T14:14:36Z</t>
+          <t>2026-10-17T13:10:02Z</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -4176,7 +4176,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Final full-cycle FEC totals and certified vote totals. One row per nominee per election. Retrieved 2026-10-09T17:06:51Z.</t>
+          <t>Final full-cycle FEC totals and certified vote totals. One row per nominee per election. Retrieved 2026-10-17T13:10:08Z.</t>
         </is>
       </c>
     </row>
@@ -6444,14 +6444,14 @@
     <row r="4" ht="120" customHeight="1">
       <c r="A4" s="85" t="inlineStr">
         <is>
-          <t>Current cycle: FEC / OpenFEC API, https://www.fec.gov/data/elections/house/PA/07/2026/, retrieved 2026-10-16T14:14:36Z</t>
+          <t>Current cycle: FEC / OpenFEC API, https://www.fec.gov/data/elections/house/PA/07/2026/, retrieved 2026-10-17T13:10:02Z</t>
         </is>
       </c>
     </row>
     <row r="5" ht="108" customHeight="1">
       <c r="A5" s="85" t="inlineStr">
         <is>
-          <t>History, finance: OpenFEC API (finance); certified results from sources/results.json, retrieved 2026-10-09T17:06:51Z</t>
+          <t>History, finance: OpenFEC API (finance); certified results from sources/results.json, retrieved 2026-10-17T13:10:08Z</t>
         </is>
       </c>
     </row>
@@ -30096,7 +30096,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cycle-to-date from each committee's latest periodic FEC report. Coverage through 2026-09-30. Retrieved 2026-10-16T14:14:36Z.</t>
+          <t>Cycle-to-date from each committee's latest periodic FEC report. Coverage through 2026-09-30. Retrieved 2026-10-17T13:10:02Z.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh FEC data 2026-10-24 13:15 UTC
</commit_message>
<xml_diff>
--- a/site/PA07_Campaign_Finance.xlsx
+++ b/site/PA07_Campaign_Finance.xlsx
@@ -3607,7 +3607,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>2026-10-23T15:03:17Z</t>
+          <t>2026-10-24T13:15:11Z</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -4176,7 +4176,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Final full-cycle FEC totals and certified vote totals. One row per nominee per election. Retrieved 2026-10-17T13:10:08Z.</t>
+          <t>Final full-cycle FEC totals and certified vote totals. One row per nominee per election. Retrieved 2026-10-24T13:15:22Z.</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4647,7 @@
         <v>1279735.82</v>
       </c>
       <c r="L10" s="59" t="n">
-        <v>654900.95</v>
+        <v>655273.84</v>
       </c>
       <c r="M10" s="59" t="n">
         <v>10853652.49</v>
@@ -6444,14 +6444,14 @@
     <row r="4" ht="120" customHeight="1">
       <c r="A4" s="85" t="inlineStr">
         <is>
-          <t>Current cycle: FEC / OpenFEC API, https://www.fec.gov/data/elections/house/PA/07/2026/, retrieved 2026-10-23T15:03:17Z</t>
+          <t>Current cycle: FEC / OpenFEC API, https://www.fec.gov/data/elections/house/PA/07/2026/, retrieved 2026-10-24T13:15:11Z</t>
         </is>
       </c>
     </row>
     <row r="5" ht="108" customHeight="1">
       <c r="A5" s="85" t="inlineStr">
         <is>
-          <t>History, finance: OpenFEC API (finance); certified results from sources/results.json, retrieved 2026-10-17T13:10:08Z</t>
+          <t>History, finance: OpenFEC API (finance); certified results from sources/results.json, retrieved 2026-10-24T13:15:22Z</t>
         </is>
       </c>
     </row>
@@ -29253,7 +29253,7 @@
       <c r="I502" s="5" t="n"/>
       <c r="J502" s="5" t="n"/>
       <c r="K502" s="33" t="n">
-        <v>654900.95</v>
+        <v>655273.84</v>
       </c>
       <c r="L502" s="34" t="n"/>
       <c r="M502" s="5" t="inlineStr">
@@ -31895,7 +31895,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cycle-to-date from each committee's latest periodic FEC report. Coverage through 2026-10-14. Retrieved 2026-10-23T15:03:17Z.</t>
+          <t>Cycle-to-date from each committee's latest periodic FEC report. Coverage through 2026-10-14. Retrieved 2026-10-24T13:15:11Z.</t>
         </is>
       </c>
     </row>

</xml_diff>